<commit_message>
Actualización automática REMAJU 2026-08-20 01:59 UTC
</commit_message>
<xml_diff>
--- a/Bloomberg_Remates_ULTIMO.xlsx
+++ b/Bloomberg_Remates_ULTIMO.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CA194"/>
+  <dimension ref="A1:CA197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -56306,6 +56306,875 @@
       <c r="BZ194" t="inlineStr"/>
       <c r="CA194" t="inlineStr"/>
     </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Remate N° 24942</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>PRIMERA CONVOCATORIA</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>REMATE SIMPLE</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>03/09/2026</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>11:59 AM</t>
+        </is>
+      </c>
+      <c r="F195" t="n">
+        <v>14</v>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>Próximo</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>02281-2023-0-2501-JR-CI-05</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>DEL SANTA</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>FENCO CUSTODIO MANUEL</t>
+        </is>
+      </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>LLANOS RONCAL SEGUNDO ALEX</t>
+        </is>
+      </c>
+      <c r="N195" t="inlineStr">
+        <is>
+          <t>EJECUCION DE GARANTIAS</t>
+        </is>
+      </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>DIECISEIS</t>
+        </is>
+      </c>
+      <c r="P195" t="inlineStr">
+        <is>
+          <t>13/05/2025</t>
+        </is>
+      </c>
+      <c r="Q195" t="inlineStr">
+        <is>
+          <t>BIEN INMUEBLE (TERRENO CERCADO) UBICADO EN PUEBLO JOVEN MIRAFLORES ALTO MZ B2 LOTE 1, ÁREA 397.85 M2, DISTRITO DE CHIMBOTE, PROVINCIA DEL SANTA, DEPARTAMENTO DE ANCASH, INSCRITO EN LA PARTIDA REGISTRAL N° P09006323 DEL REGISTRO DE PROPIEDAD INMUEBLE DE LOS REGISTROS PÚBLICOS ZONA REGISTRAL NRO. VII SEDE HUARAZ - OFICINA REGISTRAL DE CHIMBOTE.</t>
+        </is>
+      </c>
+      <c r="R195" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S195" t="n">
+        <v>380910.65</v>
+      </c>
+      <c r="T195" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="U195" t="n">
+        <v>253940.43</v>
+      </c>
+      <c r="V195" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W195" t="n">
+        <v>3.356</v>
+      </c>
+      <c r="X195" t="n">
+        <v>761.8200000000001</v>
+      </c>
+      <c r="Y195" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Z195" t="n">
+        <v>1100</v>
+      </c>
+      <c r="AA195" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="AB195" t="n">
+        <v>38091.07</v>
+      </c>
+      <c r="AC195" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="AD195" t="inlineStr"/>
+      <c r="AE195" t="inlineStr"/>
+      <c r="AF195" t="inlineStr"/>
+      <c r="AG195" t="inlineStr"/>
+      <c r="AH195" t="inlineStr"/>
+      <c r="AI195" t="inlineStr"/>
+      <c r="AJ195" t="inlineStr"/>
+      <c r="AK195" t="inlineStr"/>
+      <c r="AL195" t="inlineStr">
+        <is>
+          <t>PATRIMONIO EN FIDEICOMISO - D.LEG. N° 861 / CC MRP TRUST 2024 / NO INSCRITO EN LA SMV / DIRIGIDO A INVE</t>
+        </is>
+      </c>
+      <c r="AM195" t="inlineStr">
+        <is>
+          <t>JAVIER ANGEL ALTAMIRANO MORILLA</t>
+        </is>
+      </c>
+      <c r="AN195" t="inlineStr">
+        <is>
+          <t>ALTAMIRANO MORILLA</t>
+        </is>
+      </c>
+      <c r="AO195" t="inlineStr">
+        <is>
+          <t>Demandado</t>
+        </is>
+      </c>
+      <c r="AP195" t="inlineStr">
+        <is>
+          <t>AVISO-REMAJU</t>
+        </is>
+      </c>
+      <c r="AQ195" t="inlineStr"/>
+      <c r="AR195" t="inlineStr"/>
+      <c r="AS195" t="inlineStr"/>
+      <c r="AT195" t="inlineStr">
+        <is>
+          <t>GENERADO_POR_REMAJU_PRIMEFACES</t>
+        </is>
+      </c>
+      <c r="AU195" t="inlineStr">
+        <is>
+          <t>resolucion.pdf</t>
+        </is>
+      </c>
+      <c r="AV195" t="inlineStr">
+        <is>
+          <t>DEL SANTA</t>
+        </is>
+      </c>
+      <c r="AW195" t="inlineStr">
+        <is>
+          <t>ANCASH</t>
+        </is>
+      </c>
+      <c r="AX195" t="inlineStr">
+        <is>
+          <t>SANTA</t>
+        </is>
+      </c>
+      <c r="AY195" t="inlineStr">
+        <is>
+          <t>CHIMBOTE</t>
+        </is>
+      </c>
+      <c r="AZ195" t="inlineStr">
+        <is>
+          <t>P09006323</t>
+        </is>
+      </c>
+      <c r="BA195" t="inlineStr">
+        <is>
+          <t>TERRENOS</t>
+        </is>
+      </c>
+      <c r="BB195" t="inlineStr">
+        <is>
+          <t>PUEBLO JOVEN MIRAFLORES ALTO MZ B2 LOTE 1, ÁREA 397.85 M2, DISTRITO DE CHIMBOTE</t>
+        </is>
+      </c>
+      <c r="BC195" t="inlineStr">
+        <is>
+          <t>3.1. HIPOTECA: A) EN EL ASIENTO 00032 DE LA PARTIDA N° P09006323 DE LA ZONA REGISTRAL NRO. VII SEDE HUARAZ OFICINA REGISTRAL CHIMBOTE, SE HA INSCRITO UNA PRIMERA Y PREFERENCIAL HIPOTECA CONSTITUIDA POR SUS PROPIETARIOS GRUPO ALTAMIRANO &amp; MORILLA EIRL HASTA POR LA SUMA DE US $ 380,910.65 DÓLARES AMERICANOS, A FAVOR DEL BANCO DE CRÉDITO DEL PERÚ. 3.2. EMBARGO: B) EN EL ASIENTO 00033 DE LA PARTIDA N° P09006323 DE LA ZONA REGISTRAL NRO. VII SEDE HUARAZ OFICINA REGISTRAL CHIMBOTE, SE HA INSCRITO UN EMBARGO, HASTA POR LA SUMA DE S/. 100,000.00 SOLES, DISPUESTO POR EL JUEZ DEL NOVENO JUZGADO CIVIL DE TRUJILLO, A FAVOR DEL BANCO INTERNACIONAL DEL PERÚ, EN EL EXPEDIENTE N° 02478-2023-68-1601-JR-CI-09.</t>
+        </is>
+      </c>
+      <c r="BD195" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="BE195" t="inlineStr">
+        <is>
+          <t>1[VER]</t>
+        </is>
+      </c>
+      <c r="BF195" t="inlineStr">
+        <is>
+          <t>20/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BG195" t="inlineStr">
+        <is>
+          <t>29/08/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BH195" t="inlineStr">
+        <is>
+          <t>31/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BI195" t="inlineStr">
+        <is>
+          <t>02/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BJ195" t="inlineStr">
+        <is>
+          <t>03/09/2026 12:00:00 PM</t>
+        </is>
+      </c>
+      <c r="BK195" t="inlineStr">
+        <is>
+          <t>04/09/2026 11:59:59 AM</t>
+        </is>
+      </c>
+      <c r="BL195" t="inlineStr">
+        <is>
+          <t>07/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BM195" t="inlineStr">
+        <is>
+          <t>09/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BN195" t="inlineStr">
+        <is>
+          <t>10/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BO195" t="inlineStr">
+        <is>
+          <t>14/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BP195" t="inlineStr"/>
+      <c r="BQ195" t="inlineStr"/>
+      <c r="BR195" t="inlineStr"/>
+      <c r="BS195" t="inlineStr"/>
+      <c r="BT195" t="inlineStr"/>
+      <c r="BU195" t="inlineStr"/>
+      <c r="BV195" t="inlineStr"/>
+      <c r="BW195" t="inlineStr"/>
+      <c r="BX195" t="inlineStr"/>
+      <c r="BY195" t="inlineStr"/>
+      <c r="BZ195" t="inlineStr"/>
+      <c r="CA195" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Remate N° 24941</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>PRIMERA CONVOCATORIA</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>REMATE SIMPLE</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>03/09/2026</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>11:59 AM</t>
+        </is>
+      </c>
+      <c r="F196" t="n">
+        <v>14</v>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>Próximo</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>04377-2021-0-0401-JR-CI-03</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>AREQUIPA</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>TORREBLANCA GOMEZ CHRISTIAN OMAR</t>
+        </is>
+      </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>MARQUEZ GALARZA ERWIN ROMMEL</t>
+        </is>
+      </c>
+      <c r="N196" t="inlineStr">
+        <is>
+          <t>EJECUCION DE GARANTIAS</t>
+        </is>
+      </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="P196" t="inlineStr">
+        <is>
+          <t>23/09/2025</t>
+        </is>
+      </c>
+      <c r="Q196" t="inlineStr">
+        <is>
+          <t>CONVOCAR LA EJECUCIÓN DEL REMATE ELECTRÓNICO JUDICIAL (REM@JU) DEL BIEN INMUEBLE MATERIA DE PROCESO, SEGUIDO POR CESAR RAMIRO TORRES BERNEDO EN CONTRA DE LILA ROSA BARRAZA GOMEZ.- 2).- DATOS DE LOS BIENES OBJETO DE REMATE: URBANIZACIÓN PIEDRA SANTA (TERRENO DE OTROS FINES), DISTRITO DE YANAHUARA, PROVINCIA Y DEPARTAMENTO DE AREQUIPA, INSCRITO EN LA PARTIDA REGISTRAL N° 01160185 DEL REGISTRO DE PROPIEDAD INMUEBLE DE LA ZONA REGISTRAL XII SEDE AREQUIPA.- 3) CONVÓQUESE AUTOMÁTICAMENTE AL SEGUNDO REMATE Y SEGUIDAMENTE AL TERCER REMATE ELECTRÓNICO JUDICIAL DE SER NECESARIO, SIEMPRE Y CUANDO LA PRIMERA CONVOCATORIA HAYA SIDO DECLARADA DESIERTA A TRAVÉS DEL APLICATIVO INFORMÁTICO REM@JU POR AUSENCIA DE POSTORES O NO HAYAN INGRESADO OFERTAS SUPERIORES AL PRECIO BASE. CABE AÑADIR QUE, PARA EL DESARROLLO DEL REMATE ELECTRÓNICO JUDICIAL, EL SISTEMA REM@JU SE ENCONTRARÁ HABILITADO PARA LA COLOCACIÓN O PRESENTACIÓN DE OFERTA POR VEINTICUATRO (24) HORAS CONFORME A LEY, INICIANDO A LAS DOCE (12) HORAS DEL DÍA INDICADO COMO INICIO EN EL CRONOGRAMA DEL REMATE ELECTRÓNICO JUDICIAL Y CULMINANDO A LAS DOCE (12) HORAS DEL DÍA SIGUIENTE.</t>
+        </is>
+      </c>
+      <c r="R196" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S196" t="n">
+        <v>2969727.61</v>
+      </c>
+      <c r="T196" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="U196" t="n">
+        <v>1979818.41</v>
+      </c>
+      <c r="V196" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="W196" t="inlineStr"/>
+      <c r="X196" t="n">
+        <v>5939.46</v>
+      </c>
+      <c r="Y196" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="Z196" t="n">
+        <v>1100</v>
+      </c>
+      <c r="AA196" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="AB196" t="n">
+        <v>296972.76</v>
+      </c>
+      <c r="AC196" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="AD196" t="inlineStr"/>
+      <c r="AE196" t="inlineStr"/>
+      <c r="AF196" t="inlineStr"/>
+      <c r="AG196" t="inlineStr"/>
+      <c r="AH196" t="inlineStr"/>
+      <c r="AI196" t="inlineStr"/>
+      <c r="AJ196" t="inlineStr"/>
+      <c r="AK196" t="inlineStr"/>
+      <c r="AL196" t="inlineStr">
+        <is>
+          <t>CESAR RAMIRO TORRES BERNEDO</t>
+        </is>
+      </c>
+      <c r="AM196" t="inlineStr">
+        <is>
+          <t>LILA ROSA BARRAZA GOMEZ</t>
+        </is>
+      </c>
+      <c r="AN196" t="inlineStr">
+        <is>
+          <t>BARRAZA GOMEZ</t>
+        </is>
+      </c>
+      <c r="AO196" t="inlineStr">
+        <is>
+          <t>Demandado</t>
+        </is>
+      </c>
+      <c r="AP196" t="inlineStr">
+        <is>
+          <t>AVISO-REMAJU</t>
+        </is>
+      </c>
+      <c r="AQ196" t="inlineStr">
+        <is>
+          <t>Conforme a la partida registral 01160185: En el asiento D00003</t>
+        </is>
+      </c>
+      <c r="AR196" t="inlineStr"/>
+      <c r="AS196" t="inlineStr"/>
+      <c r="AT196" t="inlineStr">
+        <is>
+          <t>GENERADO_POR_REMAJU_PRIMEFACES</t>
+        </is>
+      </c>
+      <c r="AU196" t="inlineStr">
+        <is>
+          <t>resolucion.pdf</t>
+        </is>
+      </c>
+      <c r="AV196" t="inlineStr">
+        <is>
+          <t>AREQUIPA</t>
+        </is>
+      </c>
+      <c r="AW196" t="inlineStr">
+        <is>
+          <t>AREQUIPA</t>
+        </is>
+      </c>
+      <c r="AX196" t="inlineStr">
+        <is>
+          <t>AREQUIPA</t>
+        </is>
+      </c>
+      <c r="AY196" t="inlineStr">
+        <is>
+          <t>YANAHUARA</t>
+        </is>
+      </c>
+      <c r="AZ196" t="inlineStr">
+        <is>
+          <t>01160185</t>
+        </is>
+      </c>
+      <c r="BA196" t="inlineStr">
+        <is>
+          <t>TERRENOS</t>
+        </is>
+      </c>
+      <c r="BB196" t="inlineStr">
+        <is>
+          <t>URBANIZACIÓN PIEDRA SANTA (TERRENO DE OTROS FINES), DISTRITO DE YANAHUARA, PROVINCIA Y DEPARTAMENTO DE AREQUIPA, INSCRITO EN LA PARTIDA REGISTRAL N° 01160185 DEL REGISTRO DE PROPIEDAD INMUEBLE DE LA ZONA REGISTRAL XII SEDE AREQUIPA.-</t>
+        </is>
+      </c>
+      <c r="BC196" t="inlineStr">
+        <is>
+          <t>EN EL ASIENTO D00003 APARECE INSCRITA HIPOTECA POR S/700,000.00 INCLUYE EL INMUEBLE DE LA PARTIDA 01160186, PARA GARANTIZAR EL MUTUO OTORGADO POR LA SUMA DE S/ 443,000.00 Y US$ 18,600.00.- B) EN EL ASIENTO D00004 APARECE LA ANOTACIÓN PREVENTIVA DE CANCELACIÓN DE LOS ASIENTOS REGISTRALES D00002, C00002, D00003, POR SUPUESTA FALSEDAD DE DOCUMENTOS DENUNCIADO POR LA MUNICIPALIDAD DE YANAHUARA, SEGÚN D.LEG. 1049 MODIFICADA POR LEY 30313 LA ANOTACIÓN PREVENTIVA ES HASTA QUE SE ANOTE LA DEMANDA O MEDIDA CAUTELAR VIGENCIA DE UN AÑO DESDE EL SIENTO DE PRESENTACIÓN (28/08/2020).- E0001 LEVANTAMIENTO DE ANOTACIÓN PREVENTIVA DEL ASIENTO D0004. C0003 CANCELACION DE ASIENTO C0002. E0002 CANCELACIÓN DE ASIENTO D0002. D0005 ANOTACIÓN DE DEMANDA DE NULIDAD DE ACTO JURÍDICO ORDANADO POR EL QUINTO JUZGADO CIVIL.</t>
+        </is>
+      </c>
+      <c r="BD196" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="BE196" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BF196" t="inlineStr">
+        <is>
+          <t>20/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BG196" t="inlineStr">
+        <is>
+          <t>29/08/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BH196" t="inlineStr">
+        <is>
+          <t>31/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BI196" t="inlineStr">
+        <is>
+          <t>02/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BJ196" t="inlineStr">
+        <is>
+          <t>03/09/2026 12:00:00 PM</t>
+        </is>
+      </c>
+      <c r="BK196" t="inlineStr">
+        <is>
+          <t>04/09/2026 11:59:59 AM</t>
+        </is>
+      </c>
+      <c r="BL196" t="inlineStr">
+        <is>
+          <t>07/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BM196" t="inlineStr">
+        <is>
+          <t>09/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BN196" t="inlineStr">
+        <is>
+          <t>10/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BO196" t="inlineStr">
+        <is>
+          <t>14/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BP196" t="inlineStr"/>
+      <c r="BQ196" t="inlineStr"/>
+      <c r="BR196" t="inlineStr"/>
+      <c r="BS196" t="inlineStr"/>
+      <c r="BT196" t="inlineStr"/>
+      <c r="BU196" t="inlineStr"/>
+      <c r="BV196" t="inlineStr"/>
+      <c r="BW196" t="inlineStr"/>
+      <c r="BX196" t="inlineStr"/>
+      <c r="BY196" t="inlineStr"/>
+      <c r="BZ196" t="inlineStr"/>
+      <c r="CA196" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Remate N° 24940</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>PRIMERA CONVOCATORIA</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>REMATE SIMPLE</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>03/09/2026</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>11:59 AM</t>
+        </is>
+      </c>
+      <c r="F197" t="n">
+        <v>14</v>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>Próximo</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>03313-2019-0-0401-JR-CI-07</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>AREQUIPA</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>TORREBLANCA GOMEZ CHRISTIAN OMAR</t>
+        </is>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>TITO ZAMALLOA, LILIANA</t>
+        </is>
+      </c>
+      <c r="N197" t="inlineStr">
+        <is>
+          <t>OBLIGACION DE DAR SUMA DE DINERO</t>
+        </is>
+      </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="P197" t="inlineStr">
+        <is>
+          <t>22/08/2025</t>
+        </is>
+      </c>
+      <c r="Q197" t="inlineStr">
+        <is>
+          <t>CONVOCAR LA EJECUCIÓN DEL REMATE ELECTRÓNICO JUDICIAL (REM@JU) DE LOS BIENES INMUEBLES MATERIA DE EJECUCIÓN. 2).- DATOS DEL BIEN OBJETO DE REMATE: UBICADO EN EN LA MZ. A, LOTE 7 DE LA URBANIZACIÓN CABAÑA MARÍA DEL DISTRITO DE PAUCARPATA, PROVINCIA Y DEPARTAMENTO DE AREQUIPA, INSCRITO EN LA PARTIDA REGISTRAL NRO. 01093541 DEL REGISTRO DE PREDIOS DE LA ZONA REGISTRAL NRO. XII SEDE AREQUIPA. 3) CONVÓQUESE AUTOMÁTICAMENTE AL SEGUNDO REMATE Y SEGUIDAMENTE AL TERCER REMATE ELECTRÓNICO JUDICIAL DE SER NECESARIO, SIEMPRE Y CUANDO LA PRIMERA CONVOCATORIA HAYA SIDO DECLARADA DESIERTA A TRAVÉS DEL APLICATIVO INFORMÁTICO REM@JU POR AUSENCIA DE POSTORES O NO HAYAN INGRESADO OFERTAS SUPERIORES AL PRECIO BASE. CABE AÑADIR QUE, PARA EL DESARROLLO DEL REMATE ELECTRÓNICO JUDICIAL, EL SISTEMA REM@JU SE ENCONTRARÁ HABILITADO PARA LA COLOCACIÓN O PRESENTACIÓN DE OFERTA POR VEINTICUATRO (24) HORAS CONFORME A LEY, INICIANDO A LAS DOCE (12) HORAS DEL DÍA INDICADO COMO INICIO EN EL CRONOGRAMA DEL REMATE ELECTRÓNICO JUDICIAL Y CULMINANDO A LAS DOCE (12) HORAS DEL DÍA SIGUIENTE.</t>
+        </is>
+      </c>
+      <c r="R197" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S197" t="n">
+        <v>1047102</v>
+      </c>
+      <c r="T197" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="U197" t="n">
+        <v>698068</v>
+      </c>
+      <c r="V197" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="W197" t="inlineStr"/>
+      <c r="X197" t="n">
+        <v>2094.2</v>
+      </c>
+      <c r="Y197" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="Z197" t="n">
+        <v>1100</v>
+      </c>
+      <c r="AA197" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="AB197" t="n">
+        <v>104710.2</v>
+      </c>
+      <c r="AC197" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="AD197" t="inlineStr"/>
+      <c r="AE197" t="inlineStr"/>
+      <c r="AF197" t="inlineStr"/>
+      <c r="AG197" t="inlineStr"/>
+      <c r="AH197" t="inlineStr"/>
+      <c r="AI197" t="inlineStr"/>
+      <c r="AJ197" t="inlineStr"/>
+      <c r="AK197" t="inlineStr"/>
+      <c r="AL197" t="inlineStr"/>
+      <c r="AM197" t="inlineStr">
+        <is>
+          <t>MINIST.DE TRABAJO Y PROMOCION DEL EMPLEO / JUAN CARLOS FLORES ESPINOZA</t>
+        </is>
+      </c>
+      <c r="AN197" t="inlineStr">
+        <is>
+          <t>DEL EMPLEO</t>
+        </is>
+      </c>
+      <c r="AO197" t="inlineStr">
+        <is>
+          <t>Demandado</t>
+        </is>
+      </c>
+      <c r="AP197" t="inlineStr">
+        <is>
+          <t>HÍBRIDO-AVISO-PDF+NARR+WEB+TOTAL</t>
+        </is>
+      </c>
+      <c r="AQ197" t="inlineStr"/>
+      <c r="AR197" t="inlineStr"/>
+      <c r="AS197" t="inlineStr"/>
+      <c r="AT197" t="inlineStr">
+        <is>
+          <t>GENERADO_POR_REMAJU_PRIMEFACES</t>
+        </is>
+      </c>
+      <c r="AU197" t="inlineStr">
+        <is>
+          <t>resolucion.pdf</t>
+        </is>
+      </c>
+      <c r="AV197" t="inlineStr">
+        <is>
+          <t>AREQUIPA</t>
+        </is>
+      </c>
+      <c r="AW197" t="inlineStr">
+        <is>
+          <t>AREQUIPA</t>
+        </is>
+      </c>
+      <c r="AX197" t="inlineStr">
+        <is>
+          <t>AREQUIPA</t>
+        </is>
+      </c>
+      <c r="AY197" t="inlineStr">
+        <is>
+          <t>PAUCARPATA</t>
+        </is>
+      </c>
+      <c r="AZ197" t="inlineStr">
+        <is>
+          <t>01093541</t>
+        </is>
+      </c>
+      <c r="BA197" t="inlineStr">
+        <is>
+          <t>CASA</t>
+        </is>
+      </c>
+      <c r="BB197" t="inlineStr">
+        <is>
+          <t>UBICADO EN EN LA MZ. A, LOTE 7 DE LA URBANIZACIÓN CABAÑA MARÍA DEL DISTRITO DE PAUCARPATA, PROVINCIA Y DEPARTAMENTO DE AREQUIPA, INSCRITO EN LA PARTIDA REGISTRAL NRO. 01093541 DEL REGISTRO DE PREDIOS DE LA ZONA REGISTRAL NRO. XII SEDE AREQUIPA.</t>
+        </is>
+      </c>
+      <c r="BC197" t="inlineStr">
+        <is>
+          <t>I) ASIENTO D00002. EMBARGO EN EL ORDENADO POR EL JUEZ EL SÉTIMO JUZGADO CIVIL DE LA CORTE SUPERIOR DE JUSTICIA DE AREQUIPA, CARLOS ENRIQUE POLANCO GUTIÉRREZ HA RESUELTO CONCEDER MEDIDA CAUTELAR DE EMBARGO EN FORMA DE INSCRIPCIÓN QUE RECAE SOBRE LOS DERECHOS DE PROPIEDAD DE LLANTACENTRO GEPSA E.I.R.L. HASTA POR LA SUMA DE US$ 65,500.00 DÓLARES AMERICANOS. II) ASIENTO D00003. MEDIDA CAUTELAR DE EMBARGO. POR RESOLUCIÓN COACTIVA N° 06-2022-MTPE/4/11.01 DE FECHA 12-10-2022 EN EL EXPEDIENTE N° 1902030789.21, EL EJECUTOR COACTIVO (E) DEL MINISTERIO DE TRABAJO Y PROMOCIÓN DEL EMPLEO JUAN RICARDO PAREJA POCCORI; HA DISPUESTO TRABAR MEDIDA CAUTELAR DE EMBARGO EN FORMA DE INSCRIPCIÓN SOBRE EL INMUEBLE INSCRITO EN LA PRESENTE PARTIDA DE PROPIEDAD DE LLANTACENTRO GEPSA E.I.R.L. HASTA POR LA SUMA DE S/. 7,766.00 SOLES. III) ASIENTO D00004. AMPLIACIÓN DE MEDIDA CAUTELAR DE EMBARGO COACTIVO. POR RESOLUCIÓN COACTIVA N° 09-2024-MTPE/4/11.01 DE FECHA 27/03/2024 EXPEDIDA EN EL EXPEDIENTE N° 1902030789.21, EN EL PROCEDIMIENTO COACTIVO SOBRE PAGO DE DEUDA SEGUIDO POR EL MINISTERIO DE TRABAJO Y PROMOCIÓN DEL EMPLEO, EL EJECUTOR COACTIVO ABG. JUAN RICARDO PAREJA POCCORI, HA DISPUESTO AMPLIAR LA MEDIDA CAUTELAR DE EMBARGO EN FORMA DE INSCRIPCIÓN, INSCRITA EN EL ASIENTO D0003 DE ESTA PARTIDA HASTA POR LA SUMA DE S/. 8,693.00 SOLES.</t>
+        </is>
+      </c>
+      <c r="BD197" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="BE197" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BF197" t="inlineStr">
+        <is>
+          <t>20/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BG197" t="inlineStr">
+        <is>
+          <t>29/08/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BH197" t="inlineStr">
+        <is>
+          <t>31/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BI197" t="inlineStr">
+        <is>
+          <t>02/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BJ197" t="inlineStr">
+        <is>
+          <t>03/09/2026 12:00:00 PM</t>
+        </is>
+      </c>
+      <c r="BK197" t="inlineStr">
+        <is>
+          <t>04/09/2026 11:59:59 AM</t>
+        </is>
+      </c>
+      <c r="BL197" t="inlineStr">
+        <is>
+          <t>07/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BM197" t="inlineStr">
+        <is>
+          <t>09/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BN197" t="inlineStr">
+        <is>
+          <t>10/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BO197" t="inlineStr">
+        <is>
+          <t>14/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BP197" t="inlineStr"/>
+      <c r="BQ197" t="inlineStr"/>
+      <c r="BR197" t="inlineStr"/>
+      <c r="BS197" t="inlineStr"/>
+      <c r="BT197" t="inlineStr"/>
+      <c r="BU197" t="inlineStr"/>
+      <c r="BV197" t="inlineStr"/>
+      <c r="BW197" t="inlineStr"/>
+      <c r="BX197" t="inlineStr"/>
+      <c r="BY197" t="inlineStr"/>
+      <c r="BZ197" t="inlineStr"/>
+      <c r="CA197" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualización automática REMAJU 2026-08-20 19:12 UTC
</commit_message>
<xml_diff>
--- a/Bloomberg_Remates_ULTIMO.xlsx
+++ b/Bloomberg_Remates_ULTIMO.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CA197"/>
+  <dimension ref="A1:CA205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -57175,6 +57175,2318 @@
       <c r="BZ197" t="inlineStr"/>
       <c r="CA197" t="inlineStr"/>
     </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Remate N° 24950</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>PRIMERA CONVOCATORIA</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>REMATE SIMPLE</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>03/09/2026</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>11:59 AM</t>
+        </is>
+      </c>
+      <c r="F198" t="n">
+        <v>14</v>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>Próximo</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>00170-2025-0-1411-JR-CI-01</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>ICA</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>MAQUERA PILCOMAMANI EDWIN LUIS</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>CESAR SASIETA FAJARDO</t>
+        </is>
+      </c>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>EJECUCION DE GARANTIAS</t>
+        </is>
+      </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="P198" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="Q198" t="inlineStr">
+        <is>
+          <t>INMUEBLE UBICADO EN CALLE CONCORDIA SUB LOTE 1-B URB. SAN JORGE – DISTRITO DE PISCO Y PROVINCIA DE PISCO, DEPARTAMENTO DE ICA, INSCRITO EN LA PARTIDA REGISTRAL N°P02005316.</t>
+        </is>
+      </c>
+      <c r="R198" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S198" t="n">
+        <v>209243.39</v>
+      </c>
+      <c r="T198" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="U198" t="n">
+        <v>139495.59</v>
+      </c>
+      <c r="V198" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="W198" t="inlineStr"/>
+      <c r="X198" t="n">
+        <v>418.49</v>
+      </c>
+      <c r="Y198" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="Z198" t="n">
+        <v>550</v>
+      </c>
+      <c r="AA198" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="AB198" t="n">
+        <v>20924.34</v>
+      </c>
+      <c r="AC198" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="AD198" t="inlineStr"/>
+      <c r="AE198" t="inlineStr"/>
+      <c r="AF198" t="inlineStr"/>
+      <c r="AG198" t="inlineStr"/>
+      <c r="AH198" t="inlineStr"/>
+      <c r="AI198" t="inlineStr"/>
+      <c r="AJ198" t="inlineStr"/>
+      <c r="AK198" t="inlineStr"/>
+      <c r="AL198" t="inlineStr">
+        <is>
+          <t>TERESA JULIETA MONRROY CONISLLA / MIGUEL EDUARDO ZEGARRA PONS</t>
+        </is>
+      </c>
+      <c r="AM198" t="inlineStr">
+        <is>
+          <t>KARIME ALEJANDRA PEÑA HEREDIA</t>
+        </is>
+      </c>
+      <c r="AN198" t="inlineStr">
+        <is>
+          <t>PEÑA HEREDIA</t>
+        </is>
+      </c>
+      <c r="AO198" t="inlineStr">
+        <is>
+          <t>Demandado</t>
+        </is>
+      </c>
+      <c r="AP198" t="inlineStr">
+        <is>
+          <t>AVISO-REMAJU</t>
+        </is>
+      </c>
+      <c r="AQ198" t="inlineStr"/>
+      <c r="AR198" t="inlineStr"/>
+      <c r="AS198" t="inlineStr"/>
+      <c r="AT198" t="inlineStr">
+        <is>
+          <t>GENERADO_POR_REMAJU_PRIMEFACES</t>
+        </is>
+      </c>
+      <c r="AU198" t="inlineStr">
+        <is>
+          <t>resolucion.pdf</t>
+        </is>
+      </c>
+      <c r="AV198" t="inlineStr">
+        <is>
+          <t>ICA</t>
+        </is>
+      </c>
+      <c r="AW198" t="inlineStr">
+        <is>
+          <t>ICA</t>
+        </is>
+      </c>
+      <c r="AX198" t="inlineStr">
+        <is>
+          <t>PISCO</t>
+        </is>
+      </c>
+      <c r="AY198" t="inlineStr">
+        <is>
+          <t>PISCO</t>
+        </is>
+      </c>
+      <c r="AZ198" t="inlineStr">
+        <is>
+          <t>P02005316</t>
+        </is>
+      </c>
+      <c r="BA198" t="inlineStr">
+        <is>
+          <t>CASA</t>
+        </is>
+      </c>
+      <c r="BB198" t="inlineStr">
+        <is>
+          <t>INMUEBLE UBICADO EN CALLE CONCORDIA SUB LOTE 1-B URB. SAN JORGE – DISTRITO DE PISCO Y PROVINCIA DE PISCO, DEPARTAMENTO DE ICA, INSCRITO EN LA PARTIDA REGISTRAL N°P02005316.</t>
+        </is>
+      </c>
+      <c r="BC198" t="inlineStr">
+        <is>
+          <t>EN EL ASIENTO D00005 DE LA PARTIDA NRO. P02005316 DEL REGISTRO DE PROPIEDAD INMUEBLE DE PISCO – ZONA REGISTRAL N° XI – SEDE ICA. SE HA INSCRITO UNA HIPOTECA CONSTITUIDA POR SU PROPIETARIO EN FAVOR DE MIGUEL EDUARDO ZEGARRA PONS CASADO, CON TERESA JULIETA MONRROY CONISLLA HASTA POR EL MONTO DE S/. 200, 000.00 SOLES.</t>
+        </is>
+      </c>
+      <c r="BD198" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="BE198" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BF198" t="inlineStr">
+        <is>
+          <t>21/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BG198" t="inlineStr">
+        <is>
+          <t>30/08/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BH198" t="inlineStr">
+        <is>
+          <t>31/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BI198" t="inlineStr">
+        <is>
+          <t>02/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BJ198" t="inlineStr">
+        <is>
+          <t>03/09/2026 12:00:00 PM</t>
+        </is>
+      </c>
+      <c r="BK198" t="inlineStr">
+        <is>
+          <t>04/09/2026 11:59:59 AM</t>
+        </is>
+      </c>
+      <c r="BL198" t="inlineStr">
+        <is>
+          <t>07/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BM198" t="inlineStr">
+        <is>
+          <t>09/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BN198" t="inlineStr">
+        <is>
+          <t>10/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BO198" t="inlineStr">
+        <is>
+          <t>14/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BP198" t="inlineStr"/>
+      <c r="BQ198" t="inlineStr"/>
+      <c r="BR198" t="inlineStr"/>
+      <c r="BS198" t="inlineStr"/>
+      <c r="BT198" t="inlineStr"/>
+      <c r="BU198" t="inlineStr"/>
+      <c r="BV198" t="inlineStr"/>
+      <c r="BW198" t="inlineStr"/>
+      <c r="BX198" t="inlineStr"/>
+      <c r="BY198" t="inlineStr"/>
+      <c r="BZ198" t="inlineStr"/>
+      <c r="CA198" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Remate N° 24949</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>PRIMERA CONVOCATORIA</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>REMATE SIMPLE</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>03/09/2026</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>11:59 AM</t>
+        </is>
+      </c>
+      <c r="F199" t="n">
+        <v>14</v>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>Próximo</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>01973-2023-0-2301-JR-CI-03</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>TACNA</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>VERA ESQUIVEL, JUAN MANUEL</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>RODRIGUEZ TANTA, JORGE - EJE EJECUCION</t>
+        </is>
+      </c>
+      <c r="N199" t="inlineStr">
+        <is>
+          <t>EJECUCION DE GARANTIAS</t>
+        </is>
+      </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P199" t="inlineStr">
+        <is>
+          <t>17/06/2026</t>
+        </is>
+      </c>
+      <c r="Q199" t="inlineStr">
+        <is>
+          <t>BIEN: UBICADO EN PUEBLO JOVEN NUESTRA SEÑORA DE LA NATIVIDAD MZ. 31 LOTE 2, DEL DISTRITO, PROVINCIA Y DEPARTAMENTO DE TACNA, INSCRITO EN LA PARTIDA NRO. P20015569 DEL REGISTRO PREDIAL URBANO DE LA ZONA REGISTRAL NRO. XIII – SEDE TACNA [ÁREA DE 251.60 M2</t>
+        </is>
+      </c>
+      <c r="R199" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S199" t="n">
+        <v>345820.38</v>
+      </c>
+      <c r="T199" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="U199" t="n">
+        <v>230546.92</v>
+      </c>
+      <c r="V199" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="W199" t="inlineStr"/>
+      <c r="X199" t="n">
+        <v>691.64</v>
+      </c>
+      <c r="Y199" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="Z199" t="n">
+        <v>825</v>
+      </c>
+      <c r="AA199" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="AB199" t="n">
+        <v>34582.04</v>
+      </c>
+      <c r="AC199" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="AD199" t="inlineStr"/>
+      <c r="AE199" t="inlineStr"/>
+      <c r="AF199" t="inlineStr"/>
+      <c r="AG199" t="inlineStr"/>
+      <c r="AH199" t="inlineStr"/>
+      <c r="AI199" t="inlineStr"/>
+      <c r="AJ199" t="inlineStr"/>
+      <c r="AK199" t="inlineStr"/>
+      <c r="AL199" t="inlineStr">
+        <is>
+          <t>SCOTIABANK PERU SAA</t>
+        </is>
+      </c>
+      <c r="AM199" t="inlineStr">
+        <is>
+          <t>NANCY GUADALUPE UCHASARA CONDORI / PERCY LUCIO KENTA QUISPE</t>
+        </is>
+      </c>
+      <c r="AN199" t="inlineStr">
+        <is>
+          <t>UCHASARA CONDORI</t>
+        </is>
+      </c>
+      <c r="AO199" t="inlineStr">
+        <is>
+          <t>Demandado</t>
+        </is>
+      </c>
+      <c r="AP199" t="inlineStr">
+        <is>
+          <t>AVISO-REMAJU</t>
+        </is>
+      </c>
+      <c r="AQ199" t="inlineStr"/>
+      <c r="AR199" t="inlineStr"/>
+      <c r="AS199" t="inlineStr"/>
+      <c r="AT199" t="inlineStr">
+        <is>
+          <t>GENERADO_POR_REMAJU_PRIMEFACES</t>
+        </is>
+      </c>
+      <c r="AU199" t="inlineStr">
+        <is>
+          <t>resolucion.pdf</t>
+        </is>
+      </c>
+      <c r="AV199" t="inlineStr">
+        <is>
+          <t>TACNA</t>
+        </is>
+      </c>
+      <c r="AW199" t="inlineStr">
+        <is>
+          <t>TACNA</t>
+        </is>
+      </c>
+      <c r="AX199" t="inlineStr">
+        <is>
+          <t>TACNA</t>
+        </is>
+      </c>
+      <c r="AY199" t="inlineStr">
+        <is>
+          <t>TACNA</t>
+        </is>
+      </c>
+      <c r="AZ199" t="inlineStr">
+        <is>
+          <t>P20015569</t>
+        </is>
+      </c>
+      <c r="BA199" t="inlineStr">
+        <is>
+          <t>CASA</t>
+        </is>
+      </c>
+      <c r="BB199" t="inlineStr">
+        <is>
+          <t>UBICADO EN PUEBLO JOVEN NUESTRA SEÑORA DE LA NATIVIDAD MZ. 31 LOTE 2, DEL DISTRITO, PROVINCIA Y DEPARTAMENTO DE TACNA</t>
+        </is>
+      </c>
+      <c r="BC199" t="inlineStr">
+        <is>
+          <t>ASIENTO NRO. 00007 CONSTITUCION DE HIPOTECA LOS COPROPIETARIOS DEL PREDIO INSCRITO EN ESTA PARTIDA REGISTRAL, PERCY LUCIO KENTA QUISPE Y NANCY GUADALUPE UCHASARA CONDORI, CONSTITUYEN HIPOTECA A PLAZO INDETERMINADO A FAVOR DEL BANCO SCOTIABANK PERÚ S.A.A. CON RUC NRO. 20100043140 INSCRITO EN LA PARTIDA REGISTRAL NRO. 11008578 DEL REGISTRO DE PERSONAS JURÍDICAS DE LA OFICINA REGISTRAL DE LIMA, HASTA POR LA SUMA DE S/ 250,000.00, A FIN DE GARANTIZAR LA OBLIGACIÓN DETERMINADA DE CRÉDITO HASTA POR LA SUMA DE S/ 180,000.00, CUOTA PLAZO DE VENCIMIENTO ES DE 180 MESES; FECHA DE INSCRIPCIÓN 06/01/2016. 4.2 ASIENTO NRO. 00008 INSCRIPCIÓN EMBARGO MEDIDA CAUTELAR DE EMBARGO EN FORMA DE INSCRIPCIÓN FUERA DE PROCESO SOBRE EL 50% DE ACCCIONES Y DERECHOS QUE LE CORRESPONDE A PERCY LUCIO KENTA QUISPE, EXPEDIDA POR EL JUZGADO TRANSITORIO DE EXTINCIÓN DE DOMINIO DE LA CORTE SUPERIOR DE JUSTICIA DE TACNA, HASTA POR LA SUMA DE S/ 70,000.00 TRAMITADO EN EL EXPEDIENTE NRO. 01578-2004-51-2301-JR-PE-03, SOBRE OBLIGACIÓN DE DAR SUMA DE DINERO, A FAVOR DE SUB CAFAE DRET DEL MINISTERIO DE EDUCACIÓN; FECHA DE INSCRIPCIÓN 04/09/2019. 4.3 ASIENTO NRO. 00009 MEDIDA CAUTELAR DE EMBARGO EN FORMA DE INSCRIPCIÓN FUERA DEL PROCESO, EXPEDIDA POR EL SEGUNDO JUZGADO ESPECIALIZADO EN LO CIVIL DE LA CORTE SUPERIOR DE JUSTICIA DE TACNA, HASTA POR LA SUMA DE S/ 49,000.00 EN EL EXPEDIENTE NRO. 00275-2020-25-2301-JR-CI-02, SOBRE OBLIGACIÓN DE DAR SUMA DE DINERO, A FAVOR DE BANCO INTERNACIONAL DEL PERU – INTERBANK; FECHA DE INSCRIPCIÓN 25/12/2020</t>
+        </is>
+      </c>
+      <c r="BD199" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="BE199" t="inlineStr">
+        <is>
+          <t>1[VER]</t>
+        </is>
+      </c>
+      <c r="BF199" t="inlineStr">
+        <is>
+          <t>21/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BG199" t="inlineStr">
+        <is>
+          <t>30/08/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BH199" t="inlineStr">
+        <is>
+          <t>31/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BI199" t="inlineStr">
+        <is>
+          <t>02/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BJ199" t="inlineStr">
+        <is>
+          <t>03/09/2026 12:00:00 PM</t>
+        </is>
+      </c>
+      <c r="BK199" t="inlineStr">
+        <is>
+          <t>04/09/2026 11:59:59 AM</t>
+        </is>
+      </c>
+      <c r="BL199" t="inlineStr">
+        <is>
+          <t>07/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BM199" t="inlineStr">
+        <is>
+          <t>09/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BN199" t="inlineStr">
+        <is>
+          <t>10/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BO199" t="inlineStr">
+        <is>
+          <t>14/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BP199" t="inlineStr"/>
+      <c r="BQ199" t="inlineStr"/>
+      <c r="BR199" t="inlineStr"/>
+      <c r="BS199" t="inlineStr"/>
+      <c r="BT199" t="inlineStr"/>
+      <c r="BU199" t="inlineStr"/>
+      <c r="BV199" t="inlineStr"/>
+      <c r="BW199" t="inlineStr"/>
+      <c r="BX199" t="inlineStr"/>
+      <c r="BY199" t="inlineStr"/>
+      <c r="BZ199" t="inlineStr"/>
+      <c r="CA199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Remate N° 24948</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>PRIMERA CONVOCATORIA</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>REMATE SIMPLE</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>03/09/2026</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>11:59 AM</t>
+        </is>
+      </c>
+      <c r="F200" t="n">
+        <v>14</v>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>Próximo</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>00794-2016-0-0201-JR-CI-01</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>ANCASH</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>MANRIQUE GAMARRA KARINA</t>
+        </is>
+      </c>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>SALINAS REYES PATRICIA.</t>
+        </is>
+      </c>
+      <c r="N200" t="inlineStr">
+        <is>
+          <t>EJECUCION DE GARANTIAS</t>
+        </is>
+      </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="P200" t="inlineStr">
+        <is>
+          <t>09/01/2025</t>
+        </is>
+      </c>
+      <c r="Q200" t="inlineStr">
+        <is>
+          <t>INMUEBLE UBICADO EN LA MZ. A3, LT 1 (ACTUALMENTE JR. HUAYLAS N° 287) – CENTRO POBLADO DE VICOS, DISTRITO DE MARCARÁ, PROVINCIA DE CARHUAZ, DEPARTAMENTO DE ANCASH, CON UN ÁREA DE 183.89 M2, Y UN PERÍMETRO DE 59.60 M, INSCRITO EN LA PARTIDA N° P37026962 DE LA ZONA REGISTRAL N° VII – SEDE HUARAZ.</t>
+        </is>
+      </c>
+      <c r="R200" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S200" t="n">
+        <v>76647.64</v>
+      </c>
+      <c r="T200" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="U200" t="n">
+        <v>51098.43</v>
+      </c>
+      <c r="V200" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W200" t="n">
+        <v>3.355</v>
+      </c>
+      <c r="X200" t="n">
+        <v>153.3</v>
+      </c>
+      <c r="Y200" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Z200" t="n">
+        <v>550</v>
+      </c>
+      <c r="AA200" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="AB200" t="n">
+        <v>7664.76</v>
+      </c>
+      <c r="AC200" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="AD200" t="inlineStr"/>
+      <c r="AE200" t="inlineStr"/>
+      <c r="AF200" t="inlineStr"/>
+      <c r="AG200" t="inlineStr"/>
+      <c r="AH200" t="inlineStr"/>
+      <c r="AI200" t="inlineStr"/>
+      <c r="AJ200" t="inlineStr"/>
+      <c r="AK200" t="inlineStr"/>
+      <c r="AL200" t="inlineStr"/>
+      <c r="AM200" t="inlineStr">
+        <is>
+          <t>MARCELA AURORA LAZARO CHAUCA / ELMER ROOSVELTD VEGA LEYVA</t>
+        </is>
+      </c>
+      <c r="AN200" t="inlineStr">
+        <is>
+          <t>LAZARO CHAUCA</t>
+        </is>
+      </c>
+      <c r="AO200" t="inlineStr">
+        <is>
+          <t>Demandado</t>
+        </is>
+      </c>
+      <c r="AP200" t="inlineStr">
+        <is>
+          <t>HÍBRIDO-AVISO-PDF+NARR+WEB+TOTAL</t>
+        </is>
+      </c>
+      <c r="AQ200" t="inlineStr"/>
+      <c r="AR200" t="inlineStr"/>
+      <c r="AS200" t="inlineStr"/>
+      <c r="AT200" t="inlineStr">
+        <is>
+          <t>GENERADO_POR_REMAJU_PRIMEFACES</t>
+        </is>
+      </c>
+      <c r="AU200" t="inlineStr">
+        <is>
+          <t>resolucion.pdf</t>
+        </is>
+      </c>
+      <c r="AV200" t="inlineStr">
+        <is>
+          <t>ANCASH</t>
+        </is>
+      </c>
+      <c r="AW200" t="inlineStr">
+        <is>
+          <t>ANCASH</t>
+        </is>
+      </c>
+      <c r="AX200" t="inlineStr">
+        <is>
+          <t>CARHUAZ</t>
+        </is>
+      </c>
+      <c r="AY200" t="inlineStr">
+        <is>
+          <t>MARCARA</t>
+        </is>
+      </c>
+      <c r="AZ200" t="inlineStr">
+        <is>
+          <t>P37026962</t>
+        </is>
+      </c>
+      <c r="BA200" t="inlineStr">
+        <is>
+          <t>CASA</t>
+        </is>
+      </c>
+      <c r="BB200" t="inlineStr">
+        <is>
+          <t>INMUEBLE UBICADO EN LA MZ. A3, LT 1 (ACTUALMENTE JR. HUAYLAS N° 287) – CENTRO POBLADO DE VICOS, DISTRITO DE MARCARÁ, PROVINCIA DE CARHUAZ, DEPARTAMENTO DE ANCASH, CON UN ÁREA DE 183.89 M2, Y UN PERÍMETRO DE 59.60 M, INSCRITO EN LA PARTIDA N° P37026962 DE LA ZONA REGISTRAL N° VII – SEDE HUARAZ.</t>
+        </is>
+      </c>
+      <c r="BC200" t="inlineStr">
+        <is>
+          <t>HIPOTECA: EN EL ASIENTO 5 DE LA PARTIDA ELECTRÓNICA N° P37026962 DE LA ZONA REGISTRAL No VII – SEDE HUARAZ SE HA INSCRITO UNA HIPOTECA CONSTITUIDA POR EL BANCO DE CRÉDITO DEL PERÚ DEBIDAMENTE REPRESENTADO POR GISELLA ROXANA PARIAMACHI RODRIGUEZ Y VLADIMIR KERENSKY LÓPEZ ZORRILLA HASTA POR LA SUMA DE US$139,207.00 (CIENTO TREINTA Y NUEVE MIL DOSCIENTOS SIETE CON 00/100 DOLARES DE LOS ESTADOS UNIDOS DE NORTEAMERICA). 3.2 EMBARGO: EN EL ASIENTO 7 DE LA PARTIDA ELECTRÓNICA N° P37026962 DE LA ZONA REGISTRAL No VII – SEDE HUARAZ SE HA INSCRITO UNA MEDIDA. CAUTELAR DE EMBARGO EN FORMA DE INSCRIPCION, HASTA POR LA SUMA DE CUARENTA Y CINCO MIL CON 00/100 SOLES (S/.45,000.00) EN EL PROCESO SEGUIDO POR MIBANCO – BANCO DE LA MICROEMPRESA SA SOBRE OBLIGACIÓN DE DAR SUMA DE DINERO. EXP. N° 2016-411 EXPEDIDA POR EL JUZGADO MIXTO DE CARHUAZ, JUEZ BERNABÉ F. LEÓN PAUCAR, SECRETARIO FÉLIX FERNANDO MEJÍA SALAZAR.</t>
+        </is>
+      </c>
+      <c r="BD200" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="BE200" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BF200" t="inlineStr">
+        <is>
+          <t>21/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BG200" t="inlineStr">
+        <is>
+          <t>30/08/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BH200" t="inlineStr">
+        <is>
+          <t>31/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BI200" t="inlineStr">
+        <is>
+          <t>02/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BJ200" t="inlineStr">
+        <is>
+          <t>03/09/2026 12:00:00 PM</t>
+        </is>
+      </c>
+      <c r="BK200" t="inlineStr">
+        <is>
+          <t>04/09/2026 11:59:59 AM</t>
+        </is>
+      </c>
+      <c r="BL200" t="inlineStr">
+        <is>
+          <t>07/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BM200" t="inlineStr">
+        <is>
+          <t>09/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BN200" t="inlineStr">
+        <is>
+          <t>10/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BO200" t="inlineStr">
+        <is>
+          <t>14/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BP200" t="inlineStr"/>
+      <c r="BQ200" t="inlineStr"/>
+      <c r="BR200" t="inlineStr"/>
+      <c r="BS200" t="inlineStr"/>
+      <c r="BT200" t="inlineStr"/>
+      <c r="BU200" t="inlineStr"/>
+      <c r="BV200" t="inlineStr"/>
+      <c r="BW200" t="inlineStr"/>
+      <c r="BX200" t="inlineStr"/>
+      <c r="BY200" t="inlineStr"/>
+      <c r="BZ200" t="inlineStr"/>
+      <c r="CA200" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Remate N° 24947</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>PRIMERA CONVOCATORIA</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>REMATE SIMPLE</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>03/09/2026</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>11:59 AM</t>
+        </is>
+      </c>
+      <c r="F201" t="n">
+        <v>14</v>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>Próximo</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>00794-2016-0-0201-JR-CI-01</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>ANCASH</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>MANRIQUE GAMARRA KARINA</t>
+        </is>
+      </c>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>SALINAS REYES PATRICIA.</t>
+        </is>
+      </c>
+      <c r="N201" t="inlineStr">
+        <is>
+          <t>EJECUCION DE GARANTIAS</t>
+        </is>
+      </c>
+      <c r="O201" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="P201" t="inlineStr">
+        <is>
+          <t>09/01/2025</t>
+        </is>
+      </c>
+      <c r="Q201" t="inlineStr">
+        <is>
+          <t>INMUEBLE DENOMINADO TINCO, CON UC N° 72254 (ACTUALMENTE AV. AUGUSTO B. LEGUÍA S/N – AL COSTADO DEL CENTRO DE SALUD DE MARCARÁ), VALLE EL SANTA, SECTOR MACARÁ, DISTRITO DE MARCARÁ, PROVINCIA DE CARHUAZ, DEPARTAMENTO DE ANCASH, CON UN ÁREA DE 0.1496 HA Y UN PERÍMETRO DE 161.94 M, INSCRITO EN LA PARTIDA ELECTRÓNICA N° 02179937 DE LA ZONA REGISTRAL N° VII – SEDE HUARAZ.</t>
+        </is>
+      </c>
+      <c r="R201" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S201" t="n">
+        <v>180000</v>
+      </c>
+      <c r="T201" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="U201" t="n">
+        <v>120000</v>
+      </c>
+      <c r="V201" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W201" t="n">
+        <v>3.355</v>
+      </c>
+      <c r="X201" t="n">
+        <v>360</v>
+      </c>
+      <c r="Y201" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Z201" t="n">
+        <v>1100</v>
+      </c>
+      <c r="AA201" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="AB201" t="n">
+        <v>18000</v>
+      </c>
+      <c r="AC201" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="AD201" t="inlineStr"/>
+      <c r="AE201" t="inlineStr"/>
+      <c r="AF201" t="inlineStr"/>
+      <c r="AG201" t="inlineStr"/>
+      <c r="AH201" t="inlineStr"/>
+      <c r="AI201" t="inlineStr"/>
+      <c r="AJ201" t="inlineStr"/>
+      <c r="AK201" t="inlineStr"/>
+      <c r="AL201" t="inlineStr"/>
+      <c r="AM201" t="inlineStr">
+        <is>
+          <t>ELMER ROOSVELTD VEGA LEYVA / MARCELA AURORA LAZARO CHAUCA</t>
+        </is>
+      </c>
+      <c r="AN201" t="inlineStr">
+        <is>
+          <t>VEGA LEYVA</t>
+        </is>
+      </c>
+      <c r="AO201" t="inlineStr">
+        <is>
+          <t>Demandado</t>
+        </is>
+      </c>
+      <c r="AP201" t="inlineStr">
+        <is>
+          <t>HÍBRIDO-AVISO-PDF+NARR+WEB+TOTAL</t>
+        </is>
+      </c>
+      <c r="AQ201" t="inlineStr"/>
+      <c r="AR201" t="inlineStr"/>
+      <c r="AS201" t="inlineStr"/>
+      <c r="AT201" t="inlineStr">
+        <is>
+          <t>GENERADO_POR_REMAJU_PRIMEFACES</t>
+        </is>
+      </c>
+      <c r="AU201" t="inlineStr">
+        <is>
+          <t>resolucion.pdf</t>
+        </is>
+      </c>
+      <c r="AV201" t="inlineStr">
+        <is>
+          <t>ANCASH</t>
+        </is>
+      </c>
+      <c r="AW201" t="inlineStr">
+        <is>
+          <t>ANCASH</t>
+        </is>
+      </c>
+      <c r="AX201" t="inlineStr">
+        <is>
+          <t>CARHUAZ</t>
+        </is>
+      </c>
+      <c r="AY201" t="inlineStr">
+        <is>
+          <t>MARCARA</t>
+        </is>
+      </c>
+      <c r="AZ201" t="inlineStr">
+        <is>
+          <t>02179937</t>
+        </is>
+      </c>
+      <c r="BA201" t="inlineStr">
+        <is>
+          <t>TERRENOS</t>
+        </is>
+      </c>
+      <c r="BB201" t="inlineStr">
+        <is>
+          <t>INMUEBLE DENOMINADO TINCO, CON UC N° 72254 (ACTUALMENTE AV. AUGUSTO B. LEGUÍA S/N – AL COSTADO DEL CENTRO DE SALUD DE MARCARÁ), VALLE EL SANTA, SECTOR MACARÁ, DISTRITO DE MARCARÁ, PROVINCIA DE CARHUAZ, DEPARTAMENTO DE ANCASH, CON UN ÁREA DE 0.1496 HA Y UN PERÍMETRO DE 161.94 M, INSCRITO EN LA PARTIDA ELECTRÓNICA N° 02179937 DE LA ZONA REGISTRAL N° VII – SEDE HUARAZ.</t>
+        </is>
+      </c>
+      <c r="BC201" t="inlineStr">
+        <is>
+          <t>HIPOTECA: EN EL ASIENTO 2 DE LA PARTIDA ELECTRÓNICA N° 02179937 DE LA ZONA REGISTRAL No VII – SEDE HUARAZ SE HA INSCRITO UNA HIPOTECA CONSTITUIDA POR EL BANCO DE CRÉDITO DEL PERÚ DEBIDAMENTE REPRESENTADO POR GISELLA ROXANA PARIAMACHI RODRIGUEZ Y VLADIMIR KERENSKY LÓPEZ ZORRILLA HASTA POR LA SUMA DE US$209,440.00 (DOSCIENTOS NUEVE MIL CUATROCIENTOS CUARENTA CON 00/100 DOLARES DE LOS ESTADOS UNIDOS DE NORTEAMERICA).</t>
+        </is>
+      </c>
+      <c r="BD201" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="BE201" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BF201" t="inlineStr">
+        <is>
+          <t>21/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BG201" t="inlineStr">
+        <is>
+          <t>30/08/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BH201" t="inlineStr">
+        <is>
+          <t>31/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BI201" t="inlineStr">
+        <is>
+          <t>02/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BJ201" t="inlineStr">
+        <is>
+          <t>03/09/2026 12:00:00 PM</t>
+        </is>
+      </c>
+      <c r="BK201" t="inlineStr">
+        <is>
+          <t>04/09/2026 11:59:59 AM</t>
+        </is>
+      </c>
+      <c r="BL201" t="inlineStr">
+        <is>
+          <t>07/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BM201" t="inlineStr">
+        <is>
+          <t>09/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BN201" t="inlineStr">
+        <is>
+          <t>10/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BO201" t="inlineStr">
+        <is>
+          <t>14/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BP201" t="inlineStr"/>
+      <c r="BQ201" t="inlineStr"/>
+      <c r="BR201" t="inlineStr"/>
+      <c r="BS201" t="inlineStr"/>
+      <c r="BT201" t="inlineStr"/>
+      <c r="BU201" t="inlineStr"/>
+      <c r="BV201" t="inlineStr"/>
+      <c r="BW201" t="inlineStr"/>
+      <c r="BX201" t="inlineStr"/>
+      <c r="BY201" t="inlineStr"/>
+      <c r="BZ201" t="inlineStr"/>
+      <c r="CA201" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Remate N° 24946</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>PRIMERA CONVOCATORIA</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>REMATE SIMPLE</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>03/09/2026</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>11:59 AM</t>
+        </is>
+      </c>
+      <c r="F202" t="n">
+        <v>14</v>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Próximo</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>00918-2017-0-0401-JR-CI-01</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>AREQUIPA</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>TORREBLANCA GOMEZ CHRISTIAN OMAR</t>
+        </is>
+      </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>ROJAS MENDOZA HAYDEE MARUJA</t>
+        </is>
+      </c>
+      <c r="N202" t="inlineStr">
+        <is>
+          <t>EJECUCION DE GARANTIAS</t>
+        </is>
+      </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="P202" t="inlineStr">
+        <is>
+          <t>29/01/2026</t>
+        </is>
+      </c>
+      <c r="Q202" t="inlineStr">
+        <is>
+          <t>1) CONVOCAR LA EJECUCIÓN DEL REMATE ELECTRÓNICO JUDICIAL (REM@JU) EL BIEN INMUEBLE MATERIA DE EJECUCIÓN INSCRITO EN LA PARTIDA REGISTRAL N° 04002217. 2) DATOS DE LOS BIEN OBJETO DE REMATE: DENOMINADO LA ROSPIGLIOSI, SIGNADO CON UC02261, UBICADO EN EL SECTOR LA ROSPIGLIOSI, VALLE DE TAMBO, DEL DISTRITO DE DEAN VALDIVIA, PROVINCIA DE ISLAY, DEPARTAMENTO DE AREQUIPA, INSCRITO EN LA PARTIDA REGISTRAL NRO. 04002217 DEL REGISTRO DE PROPIEDAD INMUEBLE DE LA ZONA REGISTRAL NRO. XII SEDE AREQUIPA. 3) CONVÓQUESE AUTOMÁTICAMENTE AL SEGUNDO REMATE Y SEGUIDAMENTE AL TERCER REMATE ELECTRÓNICO JUDICIAL DE SER NECESARIO, SIEMPRE Y CUANDO LA PRIMERA CONVOCATORIA HAYA SIDO DECLARADA DESIERTA A TRAVÉS DEL APLICATIVO INFORMÁTICO REM@JU POR AUSENCIA DE POSTORES O NO HAYAN INGRESADO OFERTAS SUPERIORES AL PRECIO BASE. CABE AÑADIR QUE PARA EL DESARROLLO DEL REMATE ELECTRÓNICO JUDICIAL, EL SISTEMA REM@JU SE ENCONTRARÁ HABILITADO PARA LA COLOCACIÓN O PRESENTACIÓN DE OFERTA POR VEINTICUATRO (24) HORAS CONFORME A LEY, INICIANDO A LAS DOCE (12) HORAS DEL DÍA INDICADO COMO INICIO EN EL CRONOGRAMA DEL REMATE ELECTRÓNICO JUDICIAL Y CULMINANDO A LAS DOCE (12) HORAS DEL DÍA SIGUIENTE.</t>
+        </is>
+      </c>
+      <c r="R202" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S202" t="n">
+        <v>220539.8</v>
+      </c>
+      <c r="T202" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="U202" t="n">
+        <v>147026.53</v>
+      </c>
+      <c r="V202" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="W202" t="inlineStr"/>
+      <c r="X202" t="n">
+        <v>441.08</v>
+      </c>
+      <c r="Y202" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="Z202" t="n">
+        <v>550</v>
+      </c>
+      <c r="AA202" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="AB202" t="n">
+        <v>22053.98</v>
+      </c>
+      <c r="AC202" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="AD202" t="inlineStr"/>
+      <c r="AE202" t="inlineStr"/>
+      <c r="AF202" t="inlineStr"/>
+      <c r="AG202" t="inlineStr"/>
+      <c r="AH202" t="inlineStr"/>
+      <c r="AI202" t="inlineStr"/>
+      <c r="AJ202" t="inlineStr"/>
+      <c r="AK202" t="inlineStr"/>
+      <c r="AL202" t="inlineStr">
+        <is>
+          <t>BANCO AGROPECUARIO</t>
+        </is>
+      </c>
+      <c r="AM202" t="inlineStr">
+        <is>
+          <t>MARIA VIRGINIA ZEGARRA COAQUIRA DE RODRIGUEZ / AMADOR MANUEL RODRIGUEZ GUTIERREZ</t>
+        </is>
+      </c>
+      <c r="AN202" t="inlineStr">
+        <is>
+          <t>DE RODRIGUEZ</t>
+        </is>
+      </c>
+      <c r="AO202" t="inlineStr">
+        <is>
+          <t>Demandado</t>
+        </is>
+      </c>
+      <c r="AP202" t="inlineStr">
+        <is>
+          <t>AVISO-REMAJU</t>
+        </is>
+      </c>
+      <c r="AQ202" t="inlineStr"/>
+      <c r="AR202" t="inlineStr"/>
+      <c r="AS202" t="inlineStr"/>
+      <c r="AT202" t="inlineStr">
+        <is>
+          <t>GENERADO_POR_REMAJU_PRIMEFACES</t>
+        </is>
+      </c>
+      <c r="AU202" t="inlineStr">
+        <is>
+          <t>resolucion.pdf</t>
+        </is>
+      </c>
+      <c r="AV202" t="inlineStr">
+        <is>
+          <t>AREQUIPA</t>
+        </is>
+      </c>
+      <c r="AW202" t="inlineStr">
+        <is>
+          <t>AREQUIPA</t>
+        </is>
+      </c>
+      <c r="AX202" t="inlineStr">
+        <is>
+          <t>ISLAY</t>
+        </is>
+      </c>
+      <c r="AY202" t="inlineStr">
+        <is>
+          <t>DEAN VALDIVIA</t>
+        </is>
+      </c>
+      <c r="AZ202" t="inlineStr">
+        <is>
+          <t>04002217</t>
+        </is>
+      </c>
+      <c r="BA202" t="inlineStr">
+        <is>
+          <t>TERRENOS</t>
+        </is>
+      </c>
+      <c r="BB202" t="inlineStr">
+        <is>
+          <t>DENOMINADO LA ROSPIGLIOSI, SIGNADO CON UC02261, UBICADO EN EL SECTOR LA ROSPIGLIOSI, VALLE DE TAMBO, DEL DISTRITO DE DEAN VALDIVIA, PROVINCIA DE ISLAY, DEPARTAMENTO DE AREQUIPA, INSCRITO EN LA PARTIDA REGISTRAL NRO. 04002217 DEL REGISTRO DE PROPIEDAD INMUEBLE DE LA ZONA REGISTRAL NRO. XII SEDE AREQUIPA.</t>
+        </is>
+      </c>
+      <c r="BC202" t="inlineStr">
+        <is>
+          <t>I) ASIENTO D00013: INSCRIPCIÓN DE HIPOTECA A FAVOR DE LA CAJA MUNICIPAL DE AHORRO Y CRÉDITO DE ICA SOCIEDAD ANÓNIMA, HASTA POR LA SUMA S/. 90, 981.14 (NOVENTA MIL NOVECIENTOS OCHOCIENTOS UNO CON 14/100 SOLES). II) ASIENTO D00014: INSCRIPCIÓN DE HIPOTECA, A FAVOR DEL BANCO AGROPECUARIO HASTA POR LA SUMA DE S/. 161, 527.20 (CIENTO SESENTA Y UN MIL QUINIENTOS VEINTISIETE CON 20/100 SOLES). III) ASIENTO D00015: INSCRIPCIÓN DE EMBARGO, A FAVOR DE FINANCIERA CONFIANZA S.A.A., HASTA POR LA SUMA DE S/. 40, 500.00 (CUARENTA MIL QUINIENTOS CON 00/100 SOLES). IV) ASIENTO C00007: INSCRIPCIÓN DE COMPRA VENTA, A FAVOR DE LIDIA CCAPA SUPO (RECTIFICADA POR ASIENTO C00008)</t>
+        </is>
+      </c>
+      <c r="BD202" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="BE202" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BF202" t="inlineStr">
+        <is>
+          <t>21/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BG202" t="inlineStr">
+        <is>
+          <t>30/08/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BH202" t="inlineStr">
+        <is>
+          <t>31/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BI202" t="inlineStr">
+        <is>
+          <t>02/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BJ202" t="inlineStr">
+        <is>
+          <t>03/09/2026 12:00:00 PM</t>
+        </is>
+      </c>
+      <c r="BK202" t="inlineStr">
+        <is>
+          <t>04/09/2026 11:59:59 AM</t>
+        </is>
+      </c>
+      <c r="BL202" t="inlineStr">
+        <is>
+          <t>07/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BM202" t="inlineStr">
+        <is>
+          <t>09/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BN202" t="inlineStr">
+        <is>
+          <t>10/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BO202" t="inlineStr">
+        <is>
+          <t>14/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BP202" t="inlineStr"/>
+      <c r="BQ202" t="inlineStr"/>
+      <c r="BR202" t="inlineStr"/>
+      <c r="BS202" t="inlineStr"/>
+      <c r="BT202" t="inlineStr"/>
+      <c r="BU202" t="inlineStr"/>
+      <c r="BV202" t="inlineStr"/>
+      <c r="BW202" t="inlineStr"/>
+      <c r="BX202" t="inlineStr"/>
+      <c r="BY202" t="inlineStr"/>
+      <c r="BZ202" t="inlineStr"/>
+      <c r="CA202" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Remate N° 24945</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>PRIMERA CONVOCATORIA</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>REMATE SIMPLE</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>03/09/2026</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>11:59 AM</t>
+        </is>
+      </c>
+      <c r="F203" t="n">
+        <v>14</v>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>Próximo</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>20689-2023-0-1817-JR-CO-07</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>LIMA</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>VARILLAS SOLANO, JUAN GUSTAVO</t>
+        </is>
+      </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>CACERES CASTILLO EDWARD JESUS</t>
+        </is>
+      </c>
+      <c r="N203" t="inlineStr">
+        <is>
+          <t>EJECUCION DE GARANTIAS</t>
+        </is>
+      </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="P203" t="inlineStr">
+        <is>
+          <t>27/05/2025</t>
+        </is>
+      </c>
+      <c r="Q203" t="inlineStr">
+        <is>
+          <t>TERRENO</t>
+        </is>
+      </c>
+      <c r="R203" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S203" t="n">
+        <v>456217</v>
+      </c>
+      <c r="T203" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="U203" t="n">
+        <v>304144.67</v>
+      </c>
+      <c r="V203" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W203" t="n">
+        <v>3.355</v>
+      </c>
+      <c r="X203" t="n">
+        <v>912.4299999999999</v>
+      </c>
+      <c r="Y203" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Z203" t="n">
+        <v>1100</v>
+      </c>
+      <c r="AA203" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="AB203" t="n">
+        <v>45621.7</v>
+      </c>
+      <c r="AC203" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="AD203" t="inlineStr"/>
+      <c r="AE203" t="inlineStr"/>
+      <c r="AF203" t="inlineStr"/>
+      <c r="AG203" t="inlineStr"/>
+      <c r="AH203" t="inlineStr"/>
+      <c r="AI203" t="inlineStr"/>
+      <c r="AJ203" t="inlineStr"/>
+      <c r="AK203" t="inlineStr"/>
+      <c r="AL203" t="inlineStr">
+        <is>
+          <t>COOPERATIVA DE AHORRO Y CREDITO AELU EN LIQUIDACION</t>
+        </is>
+      </c>
+      <c r="AM203" t="inlineStr">
+        <is>
+          <t>CONFORT AVICOLA SOCIEDAD ANONIMA CERRADA</t>
+        </is>
+      </c>
+      <c r="AN203" t="inlineStr">
+        <is>
+          <t>CONFORT AVICOLA SOCIEDAD ANONIMA CERRADA</t>
+        </is>
+      </c>
+      <c r="AO203" t="inlineStr">
+        <is>
+          <t>Demandado</t>
+        </is>
+      </c>
+      <c r="AP203" t="inlineStr">
+        <is>
+          <t>AVISO-REMAJU</t>
+        </is>
+      </c>
+      <c r="AQ203" t="inlineStr"/>
+      <c r="AR203" t="inlineStr"/>
+      <c r="AS203" t="inlineStr"/>
+      <c r="AT203" t="inlineStr">
+        <is>
+          <t>GENERADO_POR_REMAJU_PRIMEFACES</t>
+        </is>
+      </c>
+      <c r="AU203" t="inlineStr">
+        <is>
+          <t>resolucion.pdf</t>
+        </is>
+      </c>
+      <c r="AV203" t="inlineStr">
+        <is>
+          <t>PUENTE PIEDRA - VENTANILLA</t>
+        </is>
+      </c>
+      <c r="AW203" t="inlineStr">
+        <is>
+          <t>LIMA</t>
+        </is>
+      </c>
+      <c r="AX203" t="inlineStr">
+        <is>
+          <t>LIMA</t>
+        </is>
+      </c>
+      <c r="AY203" t="inlineStr">
+        <is>
+          <t>PUENTE PIEDRA</t>
+        </is>
+      </c>
+      <c r="AZ203" t="inlineStr">
+        <is>
+          <t>13207258</t>
+        </is>
+      </c>
+      <c r="BA203" t="inlineStr">
+        <is>
+          <t>TERRENOS</t>
+        </is>
+      </c>
+      <c r="BB203" t="inlineStr">
+        <is>
+          <t>SUB-LOTE 5 DE LA MANZANA G CON FRENTE A LA CALLE 3, URB. LOTIZACIÓN LAS VEGAS – PRIMERA ETAPA</t>
+        </is>
+      </c>
+      <c r="BC203" t="inlineStr">
+        <is>
+          <t>B.1. EN EL ASIENTO D00004 DE LA PARTIDA NRO. 13207258 DE LOS REGISTROS PÚBLICOS DE LIMA, SE HA INSCRITO UNA HIPOTECA POR PARTE DE CONFORT AVICOLA S.A.C. A FAVOR DE COOPERATIVA DE AHORRO Y CRÉDITO AELU, HASTA POR LA SUMA DE US$ 822,200.00, EN GARANTÍA DE LAS OBLIGACIONES CONTENIDAS EN SU DOCUMENTO CONSTITUTIVO, LA ESCRITURA PÚBLICA DEL 07 DE DICIEMBRE DE 2018, OTORGADA ANTE NOTARIO DE LIMA, SERGIO ARMANDO BERROSPI POLO. B.2. EN EL ASIENTO D00005 DE LA PARTIDA NRO. 13207258 DE LOS REGISTROS PÚBLICOS DE LIMA, SE HA INSCRITO UN EMBARGO EN FORMA DE INSCRIPCIÓN POR ORDEN DEL PRIMER JUZGADO COMERCIAL DE LIMA, EXPEDIENTE NRO. 15188-2022-65-1817-JR-CO-01, POR EL MONTO DE S/ 120,000.00, DICTADA A FAVOR DE SCOTIABANK PERÚ S.A.A. CONTRA CONFORT AVICOLA S.AC.</t>
+        </is>
+      </c>
+      <c r="BD203" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="BE203" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BF203" t="inlineStr">
+        <is>
+          <t>21/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BG203" t="inlineStr">
+        <is>
+          <t>30/08/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BH203" t="inlineStr">
+        <is>
+          <t>31/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BI203" t="inlineStr">
+        <is>
+          <t>02/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BJ203" t="inlineStr">
+        <is>
+          <t>03/09/2026 12:00:00 PM</t>
+        </is>
+      </c>
+      <c r="BK203" t="inlineStr">
+        <is>
+          <t>04/09/2026 11:59:59 AM</t>
+        </is>
+      </c>
+      <c r="BL203" t="inlineStr">
+        <is>
+          <t>07/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BM203" t="inlineStr">
+        <is>
+          <t>09/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BN203" t="inlineStr">
+        <is>
+          <t>10/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BO203" t="inlineStr">
+        <is>
+          <t>14/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BP203" t="inlineStr"/>
+      <c r="BQ203" t="inlineStr"/>
+      <c r="BR203" t="inlineStr"/>
+      <c r="BS203" t="inlineStr"/>
+      <c r="BT203" t="inlineStr"/>
+      <c r="BU203" t="inlineStr"/>
+      <c r="BV203" t="inlineStr"/>
+      <c r="BW203" t="inlineStr"/>
+      <c r="BX203" t="inlineStr"/>
+      <c r="BY203" t="inlineStr"/>
+      <c r="BZ203" t="inlineStr"/>
+      <c r="CA203" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Remate N° 24944</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>PRIMERA CONVOCATORIA</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>REMATE SIMPLE</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>03/09/2026</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>11:59 AM</t>
+        </is>
+      </c>
+      <c r="F204" t="n">
+        <v>14</v>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>Próximo</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>00699-2022-0-1903-JR-CI-01</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>LORETO</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>MONCADA MOZOMBITE JOSE ITALO</t>
+        </is>
+      </c>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>GUERRA MATICORENA NADIEZDHA ELENA</t>
+        </is>
+      </c>
+      <c r="N204" t="inlineStr">
+        <is>
+          <t>EJECUCION DE GARANTIAS</t>
+        </is>
+      </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="P204" t="inlineStr">
+        <is>
+          <t>27/06/2025</t>
+        </is>
+      </c>
+      <c r="Q204" t="inlineStr">
+        <is>
+          <t>INMUEBLE UBICADO EN EL ASENTAMIENTO HUMANO AGRUPAMIENTO DE VIVIENDA EL CASTAÑAL. MZ. “Ñ”. LOTE 25 DEL DISTRITO DE SAN JUAN BAUTISTA, PROVINCIA DE MAYNAS, DEPARTAMENTO DE LORETO, INSCRITO EN LA PARTIDA ELECTRÓNICA N° P12003512 DEL REGISTRO DE PROPIEDAD INMUEBLE DE LOS REGISTROS PÚBLICOS DE LORETO</t>
+        </is>
+      </c>
+      <c r="R204" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S204" t="n">
+        <v>189920.22</v>
+      </c>
+      <c r="T204" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="U204" t="n">
+        <v>126613.48</v>
+      </c>
+      <c r="V204" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W204" t="n">
+        <v>3.355</v>
+      </c>
+      <c r="X204" t="n">
+        <v>379.84</v>
+      </c>
+      <c r="Y204" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Z204" t="n">
+        <v>1100</v>
+      </c>
+      <c r="AA204" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="AB204" t="n">
+        <v>18992.02</v>
+      </c>
+      <c r="AC204" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="AD204" t="inlineStr"/>
+      <c r="AE204" t="inlineStr"/>
+      <c r="AF204" t="inlineStr"/>
+      <c r="AG204" t="inlineStr"/>
+      <c r="AH204" t="inlineStr"/>
+      <c r="AI204" t="inlineStr"/>
+      <c r="AJ204" t="inlineStr"/>
+      <c r="AK204" t="inlineStr"/>
+      <c r="AL204" t="inlineStr">
+        <is>
+          <t>PATRIMONIO EN FIDEICOMISO - D. LEG. N* 861 / CC PERU TRUST 2022</t>
+        </is>
+      </c>
+      <c r="AM204" t="inlineStr">
+        <is>
+          <t>LUIS SEGUNDO LOPEZ TORREJON / INVERSIONES 8 SERVICIOS GENERALES HL E.!.R.L / LESI LLIOVANA CATASHUNGA AYAMBO</t>
+        </is>
+      </c>
+      <c r="AN204" t="inlineStr">
+        <is>
+          <t>LOPEZ TORREJON</t>
+        </is>
+      </c>
+      <c r="AO204" t="inlineStr">
+        <is>
+          <t>Demandado</t>
+        </is>
+      </c>
+      <c r="AP204" t="inlineStr">
+        <is>
+          <t>AVISO-REMAJU</t>
+        </is>
+      </c>
+      <c r="AQ204" t="inlineStr"/>
+      <c r="AR204" t="inlineStr"/>
+      <c r="AS204" t="inlineStr"/>
+      <c r="AT204" t="inlineStr">
+        <is>
+          <t>GENERADO_POR_REMAJU_PRIMEFACES</t>
+        </is>
+      </c>
+      <c r="AU204" t="inlineStr">
+        <is>
+          <t>resolucion.pdf</t>
+        </is>
+      </c>
+      <c r="AV204" t="inlineStr">
+        <is>
+          <t>LORETO</t>
+        </is>
+      </c>
+      <c r="AW204" t="inlineStr">
+        <is>
+          <t>LORETO</t>
+        </is>
+      </c>
+      <c r="AX204" t="inlineStr">
+        <is>
+          <t>MAYNAS</t>
+        </is>
+      </c>
+      <c r="AY204" t="inlineStr">
+        <is>
+          <t>SAN JUAN BAUTISTA</t>
+        </is>
+      </c>
+      <c r="AZ204" t="inlineStr">
+        <is>
+          <t>P12003512</t>
+        </is>
+      </c>
+      <c r="BA204" t="inlineStr">
+        <is>
+          <t>CASA</t>
+        </is>
+      </c>
+      <c r="BB204" t="inlineStr">
+        <is>
+          <t>INMUEBLE UBICADO EN EL ASENTAMIENTO HUMANO AGRUPAMIENTO DE VIVIENDAS EL CASTAÑAL. MZ. “Ñ”. LOTE 25 DEL DISTRITO DE SAN JUAN BAUTISTA</t>
+        </is>
+      </c>
+      <c r="BC204" t="inlineStr">
+        <is>
+          <t>HIPOTECA, CONSTITUIDA POR LOS TITULARES DEL BIEN, A FAVOR DE BBVA BANCO CONTINENTAL, HASTA POR LA SUMA DE $. 133,000.00 DÓLARES AMERICANOS, INSCRITO EN EL ASIENTO N° 00020 DEL RUBRO GRAVÁMENES Y CARGAS DE LA PARTIDA ELECTRÓNICA N° P12003512, TITULO INSCRITO EL 22 DE MAYO DEL 2018.-// 3.2. MODIFICACIÓN DE HIPOTECA: EN VIRTUD DE LA CESIÓN DE DERECHOS CELEBRADA POR EL BANCO BBVA PERÚ A FAVOR DE PATRIMONIO EN FIDEICOMISO -D. LEG. N° 861, CC PERÚ TRUST 2022, NO INSCRITO EN LA SMV, DIRIGIDO A INVERSIONISTAS INSTITUCIONALES, INSCRITO EN EL ASIENTO N° 00021 DEL RUBRO GRAVÁMENES Y CARGAS DE LA PARTIDA ELECTRÓNICA N° P12003512, TITULO INSCRITO EL 03 DE FEBRERO DEL 2025</t>
+        </is>
+      </c>
+      <c r="BD204" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="BE204" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BF204" t="inlineStr">
+        <is>
+          <t>21/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BG204" t="inlineStr">
+        <is>
+          <t>30/08/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BH204" t="inlineStr">
+        <is>
+          <t>31/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BI204" t="inlineStr">
+        <is>
+          <t>02/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BJ204" t="inlineStr">
+        <is>
+          <t>03/09/2026 12:00:00 PM</t>
+        </is>
+      </c>
+      <c r="BK204" t="inlineStr">
+        <is>
+          <t>04/09/2026 11:59:59 AM</t>
+        </is>
+      </c>
+      <c r="BL204" t="inlineStr">
+        <is>
+          <t>07/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BM204" t="inlineStr">
+        <is>
+          <t>09/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BN204" t="inlineStr">
+        <is>
+          <t>10/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BO204" t="inlineStr">
+        <is>
+          <t>14/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BP204" t="inlineStr"/>
+      <c r="BQ204" t="inlineStr"/>
+      <c r="BR204" t="inlineStr"/>
+      <c r="BS204" t="inlineStr"/>
+      <c r="BT204" t="inlineStr"/>
+      <c r="BU204" t="inlineStr"/>
+      <c r="BV204" t="inlineStr"/>
+      <c r="BW204" t="inlineStr"/>
+      <c r="BX204" t="inlineStr"/>
+      <c r="BY204" t="inlineStr"/>
+      <c r="BZ204" t="inlineStr"/>
+      <c r="CA204" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Remate N° 24943</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>PRIMERA CONVOCATORIA</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>REMATE SIMPLE</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>03/09/2026</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>11:59 AM</t>
+        </is>
+      </c>
+      <c r="F205" t="n">
+        <v>14</v>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>Próximo</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>00081-2018-0-0501-JR-CI-01</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>AYACUCHO</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>JUZGADO ESPECIALIZADO</t>
+        </is>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>GONZALES LLALLI ANTONIA</t>
+        </is>
+      </c>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>ARCE SILVA MARCO ANTONIO</t>
+        </is>
+      </c>
+      <c r="N205" t="inlineStr">
+        <is>
+          <t>EJECUCION DE GARANTIAS</t>
+        </is>
+      </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="P205" t="inlineStr">
+        <is>
+          <t>15/08/2025</t>
+        </is>
+      </c>
+      <c r="Q205" t="inlineStr">
+        <is>
+          <t>INMUEBLE DADO EN GARANTÍA UBICADO EN EL ASENTAMIENTO HUMANO SAN JUAN BAUTISTA MZ Ñ LT 15-A, SECTOR II DEL DISTRITO DE SAN JUAN BAUTISTA DE LA PROVINCIA DE HUAMANGA Y DEPARTAMENTO DE AYACUCHO, DE UN ÁREA DE 247.00 M2, INSCRITO EN LA PARTIDA ELECTRÓNICA N° 11072157 DE LA OFICINA REGISTRAL DE AYACUCHO</t>
+        </is>
+      </c>
+      <c r="R205" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S205" t="n">
+        <v>816355.41</v>
+      </c>
+      <c r="T205" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="U205" t="n">
+        <v>544236.9399999999</v>
+      </c>
+      <c r="V205" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="W205" t="inlineStr"/>
+      <c r="X205" t="n">
+        <v>1632.71</v>
+      </c>
+      <c r="Y205" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="Z205" t="n">
+        <v>1100</v>
+      </c>
+      <c r="AA205" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="AB205" t="n">
+        <v>81635.53999999999</v>
+      </c>
+      <c r="AC205" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="AD205" t="inlineStr"/>
+      <c r="AE205" t="inlineStr"/>
+      <c r="AF205" t="inlineStr"/>
+      <c r="AG205" t="inlineStr"/>
+      <c r="AH205" t="inlineStr"/>
+      <c r="AI205" t="inlineStr"/>
+      <c r="AJ205" t="inlineStr"/>
+      <c r="AK205" t="inlineStr"/>
+      <c r="AL205" t="inlineStr">
+        <is>
+          <t>BANCO DE CREDITO DEL PERU</t>
+        </is>
+      </c>
+      <c r="AM205" t="inlineStr">
+        <is>
+          <t>SATURNINO HUAMAN PALOMINO / MARIA ELENA HERNANDEZ SOLDEVILLA</t>
+        </is>
+      </c>
+      <c r="AN205" t="inlineStr">
+        <is>
+          <t>HUAMAN PALOMINO</t>
+        </is>
+      </c>
+      <c r="AO205" t="inlineStr">
+        <is>
+          <t>Demandado</t>
+        </is>
+      </c>
+      <c r="AP205" t="inlineStr">
+        <is>
+          <t>AVISO-REMAJU</t>
+        </is>
+      </c>
+      <c r="AQ205" t="inlineStr"/>
+      <c r="AR205" t="inlineStr"/>
+      <c r="AS205" t="inlineStr"/>
+      <c r="AT205" t="inlineStr">
+        <is>
+          <t>GENERADO_POR_REMAJU_PRIMEFACES</t>
+        </is>
+      </c>
+      <c r="AU205" t="inlineStr">
+        <is>
+          <t>resolucion.pdf</t>
+        </is>
+      </c>
+      <c r="AV205" t="inlineStr">
+        <is>
+          <t>AYACUCHO</t>
+        </is>
+      </c>
+      <c r="AW205" t="inlineStr">
+        <is>
+          <t>AYACUCHO</t>
+        </is>
+      </c>
+      <c r="AX205" t="inlineStr">
+        <is>
+          <t>HUAMANGA</t>
+        </is>
+      </c>
+      <c r="AY205" t="inlineStr">
+        <is>
+          <t>AYACUCHO</t>
+        </is>
+      </c>
+      <c r="AZ205" t="inlineStr">
+        <is>
+          <t>11072157</t>
+        </is>
+      </c>
+      <c r="BA205" t="inlineStr">
+        <is>
+          <t>CASA</t>
+        </is>
+      </c>
+      <c r="BB205" t="inlineStr">
+        <is>
+          <t>INMUEBLE DADO EN GARANTÍA UBICADO EN EL ASENTAMIENTO HUMANO SAN JUAN BAUTISTA MZ Ñ LT 15-A, SECTOR II DEL DISTRITO DE SAN JUAN BAUTISTA DE LA PROVINCIA DE HUAMANGA Y DEPARTAMENTO DE AYACUCHO, DE UN ÁREA DE 247.00 M2</t>
+        </is>
+      </c>
+      <c r="BC205" t="inlineStr">
+        <is>
+          <t>MINUTA 31/12/2013, BLOQUEO REGISTRAL: SE PROCEDE CON EL BLOQUEO REGISTRAL SOBRE LA PRESENTE PARTIDA, POR EL TÉRMINO DE 60 DÍAS HÁBILES CONTADOS A PARTIR DE LA PRESENTE ANOTACIÓN, POR HABERLO SOLICITADO ASÍ EL NOTARIO PÚBLICO DE AYACUCHO, DR. JOSÉ HINOSTROZA AUCASIME, MEDIANTE OFICIO 468-2013-NJHA/AYACUCHO DEL 31.12.2013, SUSTENTADO EN LA MINUTA DE GARANTÍA HIPOTECARIA DEL 31.12.2013 QUE OTORGAN LOS PROPIETARIOS SATURNINO HUAMAN PALOMINO Y MARIA ELENA HERNANDEZ SOLDEVILLA EN FAVOR DE LA COOPERATIVA DE AHORRO Y CREDITO SANTA MARIA MAGDALENA LTDA. 219, HASTA POR LA SUMA DE US$. 201, 470.02 DÓLARES AMERICANOS EN RESPALDO DE UNA LÍNEA DE CRÉDITO OTORGADA A SU FAVOR HASTA POR LA SUMA DE S/. 350,000.00 NUEVOS SOLES. EMBARGO: EL SEÑOR JUEZ DEL 20 JUZGADO ESPECIALIZADO EN LO CIVIL DE HUAMANGA, DR. CARLOS MANUEL VALDIVIA RODRÍGUEZ, CON INTERVENCIÓN DEL SECRETARIO JUDICIAL MANUEL CONDE VILCA, HA RESUELTO TRABAR MEDIDA CAUTELAR DE EMBARGO EN FORMA DE INSCRIPCIÓN SOBRE EL INMUEBLE INSCRITO EN ESTA PARTIDA DE PROPIEDAD DE LOS DEMANDADOS MARÍA ELENA HERNÁNDEZ SOLDEVILLA Y SATURNINO HUAMÁN PALOMINO, HASTA POR LA SUMA DE S/. 50, 000.00 SOLES, CONFORME ASÍ FLUYE DE LA RESOLUCIÓN N° TRES DEL 12.05.2017 DEL CUADERNO DE MEDIDA CAUTELAR DEL EXPEDIENTE N° 00549-2017-26-0501-JR-CL-02 INCOADO POR LA CAJA MUNICIPAL DE AHORRO Y CRÉDITO DE ICA S.A., CONTENIDA EN LOS PARTES JUDICIALES CERTIFICADOS EL 31.05.2017 POR EL CITADO SECRETARIO JUDICIAL Y REMITIDOS MEDIANTE OFICIO N° 0382-2017 – EXPEDIENTE N° 549-2017-26-0501-JR-CL-02-2JECH-CSJAY/PJ DEL 31.05.2017.</t>
+        </is>
+      </c>
+      <c r="BD205" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="BE205" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BF205" t="inlineStr">
+        <is>
+          <t>21/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BG205" t="inlineStr">
+        <is>
+          <t>30/08/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BH205" t="inlineStr">
+        <is>
+          <t>31/08/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BI205" t="inlineStr">
+        <is>
+          <t>02/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BJ205" t="inlineStr">
+        <is>
+          <t>03/09/2026 12:00:00 PM</t>
+        </is>
+      </c>
+      <c r="BK205" t="inlineStr">
+        <is>
+          <t>04/09/2026 11:59:59 AM</t>
+        </is>
+      </c>
+      <c r="BL205" t="inlineStr">
+        <is>
+          <t>07/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BM205" t="inlineStr">
+        <is>
+          <t>09/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BN205" t="inlineStr">
+        <is>
+          <t>10/09/2026 00:00:00 AM</t>
+        </is>
+      </c>
+      <c r="BO205" t="inlineStr">
+        <is>
+          <t>14/09/2026 23:59:59 PM</t>
+        </is>
+      </c>
+      <c r="BP205" t="inlineStr"/>
+      <c r="BQ205" t="inlineStr"/>
+      <c r="BR205" t="inlineStr"/>
+      <c r="BS205" t="inlineStr"/>
+      <c r="BT205" t="inlineStr"/>
+      <c r="BU205" t="inlineStr"/>
+      <c r="BV205" t="inlineStr"/>
+      <c r="BW205" t="inlineStr"/>
+      <c r="BX205" t="inlineStr"/>
+      <c r="BY205" t="inlineStr"/>
+      <c r="BZ205" t="inlineStr"/>
+      <c r="CA205" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>